<commit_message>
Atualiza arquivos gerados com parciais da rodada 13
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
@@ -61,12 +61,12 @@
     <t>Jogo 2 (JG2)</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>Bandoleros FCS</t>
   </si>
   <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Jogo 3 (JG3)</t>
   </si>
   <si>
@@ -79,10 +79,10 @@
     <t>Jogo 4 (JG4)</t>
   </si>
   <si>
+    <t>cartola scheuer17</t>
+  </si>
+  <si>
     <t>TEAM LOPES 99</t>
-  </si>
-  <si>
-    <t>cartola scheuer17</t>
   </si>
 </sst>
 </file>
@@ -483,10 +483,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>108.52</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>105.72</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>2.799999999999997</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -524,16 +524,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>105.72</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>108.52</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-2.799999999999997</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -589,10 +589,10 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -601,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>94.47</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>92.62</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1.849999999999994</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -630,16 +630,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>92.62</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>94.47</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-1.849999999999994</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -695,10 +695,10 @@
         <v>17</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -707,13 +707,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>136.52</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>111.22</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>25.30000000000001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -736,16 +736,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>111.22</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>136.52</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-25.30000000000001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -801,10 +801,10 @@
         <v>20</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -813,13 +813,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>97.62</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>87.92</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>9.700000000000003</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -842,16 +842,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>87.92</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>97.62</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>-9.700000000000003</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualiza Parciais Rodada 13
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
@@ -52,10 +52,10 @@
     <t>Jogo 1 (JG1)</t>
   </si>
   <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
     <t>lsauer fc</t>
-  </si>
-  <si>
-    <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
     <t>Jogo 2 (JG2)</t>
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>108.52</v>
+        <v>113.79</v>
       </c>
       <c r="H2">
-        <v>105.72</v>
+        <v>108.59</v>
       </c>
       <c r="I2">
-        <v>2.799999999999997</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -527,13 +527,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>105.72</v>
+        <v>108.59</v>
       </c>
       <c r="H3">
-        <v>108.52</v>
+        <v>113.79</v>
       </c>
       <c r="I3">
-        <v>-2.799999999999997</v>
+        <v>-5.200000000000003</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -601,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>94.47</v>
+        <v>117.54</v>
       </c>
       <c r="H2">
-        <v>92.62</v>
+        <v>93.89</v>
       </c>
       <c r="I2">
-        <v>1.849999999999994</v>
+        <v>23.65000000000001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -633,13 +633,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>92.62</v>
+        <v>93.89</v>
       </c>
       <c r="H3">
-        <v>94.47</v>
+        <v>117.54</v>
       </c>
       <c r="I3">
-        <v>-1.849999999999994</v>
+        <v>-23.65000000000001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -707,13 +707,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>136.52</v>
+        <v>136.59</v>
       </c>
       <c r="H2">
-        <v>111.22</v>
+        <v>111.29</v>
       </c>
       <c r="I2">
-        <v>25.30000000000001</v>
+        <v>25.3</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -739,13 +739,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>111.22</v>
+        <v>111.29</v>
       </c>
       <c r="H3">
-        <v>136.52</v>
+        <v>136.59</v>
       </c>
       <c r="I3">
-        <v>-25.30000000000001</v>
+        <v>-25.3</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -813,13 +813,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>97.62</v>
+        <v>106.39</v>
       </c>
       <c r="H2">
-        <v>87.92</v>
+        <v>97.79000000000001</v>
       </c>
       <c r="I2">
-        <v>9.700000000000003</v>
+        <v>8.599999999999994</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -845,13 +845,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>87.92</v>
+        <v>97.79000000000001</v>
       </c>
       <c r="H3">
-        <v>97.62</v>
+        <v>106.39</v>
       </c>
       <c r="I3">
-        <v>-9.700000000000003</v>
+        <v>-8.599999999999994</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 13
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>113.79</v>
+        <v>113.7900390625</v>
       </c>
       <c r="H2">
-        <v>108.59</v>
+        <v>108.58984375</v>
       </c>
       <c r="I2">
-        <v>5.200000000000003</v>
+        <v>5.2001953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -527,13 +527,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>108.59</v>
+        <v>108.58984375</v>
       </c>
       <c r="H3">
-        <v>113.79</v>
+        <v>113.7900390625</v>
       </c>
       <c r="I3">
-        <v>-5.200000000000003</v>
+        <v>-5.2001953125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -601,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>117.54</v>
+        <v>117.5400390625</v>
       </c>
       <c r="H2">
-        <v>93.89</v>
+        <v>93.89013671875</v>
       </c>
       <c r="I2">
-        <v>23.65000000000001</v>
+        <v>23.64990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -633,13 +633,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>93.89</v>
+        <v>93.89013671875</v>
       </c>
       <c r="H3">
-        <v>117.54</v>
+        <v>117.5400390625</v>
       </c>
       <c r="I3">
-        <v>-23.65000000000001</v>
+        <v>-23.64990234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -707,13 +707,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>136.59</v>
+        <v>136.58984375</v>
       </c>
       <c r="H2">
-        <v>111.29</v>
+        <v>111.2900390625</v>
       </c>
       <c r="I2">
-        <v>25.3</v>
+        <v>25.2998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -739,13 +739,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>111.29</v>
+        <v>111.2900390625</v>
       </c>
       <c r="H3">
-        <v>136.59</v>
+        <v>136.58984375</v>
       </c>
       <c r="I3">
-        <v>-25.3</v>
+        <v>-25.2998046875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -813,13 +813,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>106.39</v>
+        <v>106.39013671875</v>
       </c>
       <c r="H2">
-        <v>97.79000000000001</v>
+        <v>97.7900390625</v>
       </c>
       <c r="I2">
-        <v>8.599999999999994</v>
+        <v>8.60009765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -845,13 +845,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>97.79000000000001</v>
+        <v>97.7900390625</v>
       </c>
       <c r="H3">
-        <v>106.39</v>
+        <v>106.39013671875</v>
       </c>
       <c r="I3">
-        <v>-8.599999999999994</v>
+        <v>-8.60009765625</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>

<commit_message>
Resultado Final Rodada 14
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_3.xlsx
@@ -79,10 +79,10 @@
     <t>Jogo 4 (JG4)</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
     <t>cartola scheuer17</t>
-  </si>
-  <si>
-    <t>TEAM LOPES 99</t>
   </si>
 </sst>
 </file>
@@ -483,10 +483,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>113.7900390625</v>
+        <v>190.740234375</v>
       </c>
       <c r="H2">
-        <v>108.58984375</v>
+        <v>157.869873046875</v>
       </c>
       <c r="I2">
-        <v>5.2001953125</v>
+        <v>32.870361328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -524,16 +524,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>108.58984375</v>
+        <v>157.869873046875</v>
       </c>
       <c r="H3">
-        <v>113.7900390625</v>
+        <v>190.740234375</v>
       </c>
       <c r="I3">
-        <v>-5.2001953125</v>
+        <v>-32.870361328125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -589,10 +589,10 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -601,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>117.5400390625</v>
+        <v>170.679931640625</v>
       </c>
       <c r="H2">
-        <v>93.89013671875</v>
+        <v>142.47021484375</v>
       </c>
       <c r="I2">
-        <v>23.64990234375</v>
+        <v>28.209716796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -630,16 +630,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>93.89013671875</v>
+        <v>142.47021484375</v>
       </c>
       <c r="H3">
-        <v>117.5400390625</v>
+        <v>170.679931640625</v>
       </c>
       <c r="I3">
-        <v>-23.64990234375</v>
+        <v>-28.209716796875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -704,16 +704,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>136.58984375</v>
+        <v>182.639892578125</v>
       </c>
       <c r="H2">
-        <v>111.2900390625</v>
+        <v>158.340087890625</v>
       </c>
       <c r="I2">
-        <v>25.2998046875</v>
+        <v>24.2998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -727,10 +727,10 @@
         <v>18</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -739,13 +739,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>111.2900390625</v>
+        <v>158.340087890625</v>
       </c>
       <c r="H3">
-        <v>136.58984375</v>
+        <v>182.639892578125</v>
       </c>
       <c r="I3">
-        <v>-25.2998046875</v>
+        <v>-24.2998046875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -810,16 +810,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>106.39013671875</v>
+        <v>159.840087890625</v>
       </c>
       <c r="H2">
-        <v>97.7900390625</v>
+        <v>158.27001953125</v>
       </c>
       <c r="I2">
-        <v>8.60009765625</v>
+        <v>1.570068359375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -833,10 +833,10 @@
         <v>21</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -845,13 +845,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>97.7900390625</v>
+        <v>158.27001953125</v>
       </c>
       <c r="H3">
-        <v>106.39013671875</v>
+        <v>159.840087890625</v>
       </c>
       <c r="I3">
-        <v>-8.60009765625</v>
+        <v>-1.570068359375</v>
       </c>
       <c r="J3">
         <v>2</v>

</xml_diff>